<commit_message>
Update data files - Bot run at 2026-09-13 18:00:07 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>481</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00481</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-13 23:00:53 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001052</v>
+        <v>0.001056</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00481</v>
+        <v>0.00476</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-12T22:02:35.081613</t>
+          <t>2026-09-13T23:00:41.836290</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-14 01:26:03 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>467</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000934</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-14 06:51:53 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>469</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000938</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-14 19:07:41 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001583333333333333</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-14 22:40:27 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -937,16 +937,16 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>488</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>0.001626666666666667</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -988,16 +988,16 @@
         <v>200000</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>499</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>0.002495</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1039,16 +1039,16 @@
         <v>200000</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>0.00256</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1141,16 +1141,16 @@
         <v>500000</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>476</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>0.000952</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-15 01:16:55 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>528</v>
+        <v>648</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001056</v>
+        <v>0.001296</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00476</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>467</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000934</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>469</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000938</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001583333333333333</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -937,20 +937,20 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>488</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.001626666666666667</v>
+        <v>0</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -988,20 +988,20 @@
         <v>200000</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>499</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0.002495</v>
+        <v>0</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -1039,20 +1039,20 @@
         <v>200000</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>512</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0.00256</v>
+        <v>0</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>
@@ -1141,20 +1141,20 @@
         <v>500000</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0.000952</v>
+        <v>0</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-13T23:00:41.836290</t>
+          <t>2026-09-15T01:16:45.563850</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-15 06:32:16 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-15 17:33:30 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>468</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000936</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-16 14:18:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>648</v>
+        <v>520</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001296</v>
+        <v>0.00104</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>468</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000936</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-15T01:16:45.563850</t>
+          <t>2026-09-16T14:18:09.400279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-16 18:20:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>473</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00473</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-17 19:11:30 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>520</v>
+        <v>470</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00104</v>
+        <v>0.00094</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00473</v>
+        <v>0.0047</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-16T14:18:09.400279</t>
+          <t>2026-09-17T19:11:22.837366</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-18 18:10:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>486</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000972</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>568</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001136</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 01:31:23 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00094</v>
+        <v>0.000946</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0047</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>486</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000972</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>568</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001136</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-17T19:11:22.837366</t>
+          <t>2026-09-19T01:31:18.156882</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 07:10:35 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>468</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00468</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 18:45:18 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001086</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-19 23:23:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>496</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000992</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-20 06:52:31 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000946</v>
+        <v>0.00094</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>468</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00468</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>543</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001086</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>496</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000992</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-19T01:31:18.156882</t>
+          <t>2026-09-20T06:52:23.340671</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-20 18:59:01 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>514</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00514</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-20 23:25:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>465</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001008</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-21 06:56:02 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00094</v>
+        <v>0.000938</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>514</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00514</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001008</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-20T06:52:23.340671</t>
+          <t>2026-09-21T06:55:57.034430</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-21 19:09:39 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>466</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00466</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-21 22:45:28 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001008</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>664</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001328</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-22 17:13:10 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000938</v>
+        <v>0.00096</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>466</v>
+        <v>504</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00466</v>
+        <v>0.00504</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001008</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>664</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001328</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-21T06:55:57.034430</t>
+          <t>2026-09-22T17:12:58.999567</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-22 23:11:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>536</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001072</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>506</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001012</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-23 07:33:45 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>466</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001553333333333333</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-23 17:56:43 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00096</v>
+        <v>0.000954</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>504</v>
+        <v>477</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00504</v>
+        <v>0.00477</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>536</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001072</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>506</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001012</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>466</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001553333333333333</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-22T17:12:58.999567</t>
+          <t>2026-09-23T17:56:32.504859</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-23 23:54:19 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>477</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000954</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000942</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-24 18:36:33 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>477</v>
+        <v>465</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000954</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>477</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00477</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>477</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000954</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000942</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-23T17:56:32.504859</t>
+          <t>2026-09-24T18:36:25.628993</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-25 00:42:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>470</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.0047</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-26 01:52:25 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>465</v>
+        <v>510</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0.00102</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0047</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-24T18:36:25.628993</t>
+          <t>2026-09-26T01:52:22.504323</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-26 22:32:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>502</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00502</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>465</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-27 06:57:40 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>510</v>
+        <v>482</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00102</v>
+        <v>0.000964</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00502</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-26T01:52:22.504323</t>
+          <t>2026-09-27T06:57:35.429696</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-27 17:37:27 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00482</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-27 23:53:48 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.00095</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-28 11:33:15 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>482</v>
+        <v>576</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000964</v>
+        <v>0.001152</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>482</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00482</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00095</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-27T06:57:35.429696</t>
+          <t>2026-09-28T11:33:07.772125</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-28 19:27:17 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>505</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00505</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001008</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-28 23:53:39 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000944</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001763333333333333</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-29 11:30:43 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -937,16 +937,16 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>575</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>0.001916666666666667</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-30 00:42:05 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>576</v>
+        <v>473</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001152</v>
+        <v>0.000946</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00505</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001008</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000944</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>529</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001763333333333333</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -937,20 +937,20 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>575</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.001916666666666667</v>
+        <v>0</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-28T11:33:07.772125</t>
+          <t>2026-09-30T00:41:57.946993</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-30 12:55:57 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>493</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00493</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>493</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.0009859999999999999</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-30 18:19:40 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>505</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.00101</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>476</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001586666666666667</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-30 22:30:11 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -937,16 +937,16 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>0.001573333333333333</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-01 01:30:16 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000946</v>
+        <v>0.000944</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>493</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00493</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>493</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0009859999999999999</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00101</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001586666666666667</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -937,20 +937,20 @@
         <v>300000</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.001573333333333333</v>
+        <v>0</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-30T00:41:57.946993</t>
+          <t>2026-10-01T01:30:08.371130</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-02 06:01:37 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000944</v>
+        <v>0.000956</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-01T01:30:08.371130</t>
+          <t>2026-10-02T06:01:32.238382</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-02 13:01:36 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>493</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00493</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>493</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.0009859999999999999</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-02 18:37:24 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>483</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000966</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-03 07:48:47 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>478</v>
+        <v>786</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000956</v>
+        <v>0.001572</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>493</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00493</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>493</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0009859999999999999</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>483</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000966</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-02T06:01:32.238382</t>
+          <t>2026-10-03T07:48:37.993675</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-03 23:37:19 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>473</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00473</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-04 11:14:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>786</v>
+        <v>472</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001572</v>
+        <v>0.000944</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00473</v>
+        <v>0.00472</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-03T07:48:37.993675</t>
+          <t>2026-10-04T11:14:03.252233</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-04 19:21:54 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>476</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000952</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-05 01:10:14 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000944</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-05 07:32:49 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>687</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.00229</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-05 23:07:01 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000944</v>
+        <v>0.000954</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00472</v>
+        <v>0.00464</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000952</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000944</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>687</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.00229</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-04T11:14:03.252233</t>
+          <t>2026-10-05T23:06:51.897509</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-06 17:05:10 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>483</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000966</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000944</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-07 01:17:02 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000954</v>
+        <v>0.0009479999999999999</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>464</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00464</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>483</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000966</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000944</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-05T23:06:51.897509</t>
+          <t>2026-10-07T01:16:54.959276</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-07 07:36:28 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>466</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00466</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-08 07:08:34 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009479999999999999</v>
+        <v>0.000936</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>466</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00466</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-07T01:16:54.959276</t>
+          <t>2026-10-08T07:08:24.459702</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-08 14:48:26 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>470</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.0047</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>516</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001032</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-09 01:03:32 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>502</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001004</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-09 07:51:14 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000936</v>
+        <v>0.000932</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0047</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>516</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001032</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001004</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-08T07:08:24.459702</t>
+          <t>2026-10-09T07:51:09.198105</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-10 06:15:20 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00472</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-10 17:42:51 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000932</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00472</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-09T07:51:09.198105</t>
+          <t>2026-10-10T17:42:41.668903</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-11 06:14:26 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>479</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00479</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-11 18:20:48 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0.0009479999999999999</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>479</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00479</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-10T17:42:41.668903</t>
+          <t>2026-10-11T18:20:38.683442</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-13 01:10:05 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>474</v>
+        <v>502</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009479999999999999</v>
+        <v>0.001004</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-11T18:20:38.683442</t>
+          <t>2026-10-13T01:09:57.274479</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-14 05:56:27 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>502</v>
+        <v>487</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001004</v>
+        <v>0.000974</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-13T01:09:57.274479</t>
+          <t>2026-10-14T05:56:19.393078</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-14 11:33:05 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>467</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00467</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-14 23:46:46 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.00096</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>469</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000938</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-15 03:55:48 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>499</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001663333333333333</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-15 18:31:29 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>487</v>
+        <v>465</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000974</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>467</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00467</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00096</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>469</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000938</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>499</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001663333333333333</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-14T05:56:19.393078</t>
+          <t>2026-10-15T18:31:21.719767</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-15 22:00:51 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00512</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>509</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.001018</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-16 11:01:30 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>583</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001166</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-16 18:57:34 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0.000954</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>512</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00512</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>509</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.001018</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>583</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001166</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-15T18:31:21.719767</t>
+          <t>2026-10-16T18:57:26.443244</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-17 09:05:21 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>587</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00587</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-17 19:06:33 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>477</v>
+        <v>465</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000954</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>587</v>
+        <v>473</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00587</v>
+        <v>0.00473</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-16T18:57:26.443244</t>
+          <t>2026-10-17T19:06:28.546059</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-17 23:52:23 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000942</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000944</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-18 08:42:51 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>746</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.002486666666666667</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-18 19:19:21 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0.000946</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>473</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00473</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000942</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>472</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000944</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>746</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.002486666666666667</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-17T19:06:28.546059</t>
+          <t>2026-10-18T19:19:13.873899</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-20 05:53:45 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000946</v>
+        <v>0.00095</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-18T19:19:13.873899</t>
+          <t>2026-10-20T05:53:42.209829</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-20 11:10:51 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>479</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00479</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>525</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.00105</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-20 23:02:48 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000964</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-21 18:11:35 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00095</v>
+        <v>0.000946</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>479</v>
+        <v>467</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00479</v>
+        <v>0.00467</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>525</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00105</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>482</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000964</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-20T05:53:42.209829</t>
+          <t>2026-10-21T18:11:24.084868</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-23 17:47:25 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000946</v>
+        <v>0.0009479999999999999</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00467</v>
+        <v>0.00472</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-21T18:11:24.084868</t>
+          <t>2026-10-23T17:47:15.694665</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-23 23:56:39 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000942</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>469</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.000938</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-24 09:01:40 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>580</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.001933333333333333</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-25 14:30:44 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009479999999999999</v>
+        <v>0.000946</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>472</v>
+        <v>490</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00472</v>
+        <v>0.0049</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000942</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>469</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000938</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>580</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.001933333333333333</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-23T17:47:15.694665</t>
+          <t>2026-10-25T14:30:33.088354</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-25 23:28:13 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>469</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000938</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-26 01:34:09 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -682,16 +682,16 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>562</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.001124</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-26 07:34:50 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -886,16 +886,16 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>687</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.00229</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-26 14:58:28 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>473</v>
+        <v>494</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000946</v>
+        <v>0.0009879999999999999</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>490</v>
+        <v>479</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0049</v>
+        <v>0.00479</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>469</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000938</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -682,20 +682,20 @@
         <v>500000</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>562</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.001124</v>
+        <v>0</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -886,20 +886,20 @@
         <v>300000</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>687</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.00229</v>
+        <v>0</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-25T14:30:33.088354</t>
+          <t>2026-10-26T14:58:19.269456</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-28 19:00:37 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>494</v>
+        <v>472</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009879999999999999</v>
+        <v>0.000944</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>479</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00479</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-26T14:58:19.269456</t>
+          <t>2026-10-28T19:00:27.301309</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-30 01:44:01 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000944</v>
+        <v>0.000954</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-28T19:00:27.301309</t>
+          <t>2026-10-30T01:43:53.824578</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-30 23:58:22 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00471</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000942</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-31 05:20:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000954</v>
+        <v>0.000966</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00471</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -631,20 +631,20 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>471</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.000942</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-30T01:43:53.824578</t>
+          <t>2026-10-31T05:20:03.099938</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-31 11:05:05 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00504</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>